<commit_message>
Corriger les erreurs de validation ConceptMap et l'affichage SQL du mapping 7ff0e498966d321cb5d71964abdfe09eec4de72a
</commit_message>
<xml_diff>
--- a/fix-target-codes-and-display/ig/FRAllergyIntoleranceLMCDAFHIR.xlsx
+++ b/fix-target-codes-and-display/ig/FRAllergyIntoleranceLMCDAFHIR.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="84">
   <si>
     <t>Property</t>
   </si>
@@ -61,7 +61,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-23T21:45:18+00:00</t>
+    <t>2026-08-24T13:13:01+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -160,15 +160,12 @@
     <t>FRLMAllergyIntolerance.period.onsetDate</t>
   </si>
   <si>
-    <t>Observation.effectiveTime.low</t>
+    <t>source-is-narrower-than-target</t>
   </si>
   <si>
     <t>FRLMAllergyIntolerance.period.endDate</t>
   </si>
   <si>
-    <t>Observation.effectiveTime.high</t>
-  </si>
-  <si>
     <t>FRLMAllergyIntolerance.agentOrAllergen</t>
   </si>
   <si>
@@ -226,10 +223,10 @@
     <t>AllergyIntolerance.onset[x]</t>
   </si>
   <si>
-    <t>AllergyIntolerance.onset[x].start</t>
-  </si>
-  <si>
-    <t>AllergyIntolerance.onset[x].end</t>
+    <t>AllergyIntolerance.onset[x]:onsetPeriod.start</t>
+  </si>
+  <si>
+    <t>AllergyIntolerance.onset[x]:onsetPeriod.end</t>
   </si>
   <si>
     <t>AllergyIntolerance.reaction</t>
@@ -647,10 +644,10 @@
       </c>
       <c r="B9" s="2"/>
       <c r="C9" t="s" s="2">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E9" s="2"/>
     </row>
@@ -660,62 +657,62 @@
       </c>
       <c r="B10" s="2"/>
       <c r="C10" t="s" s="2">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E10" s="2"/>
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B11" s="2"/>
       <c r="C11" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E11" s="2"/>
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B12" s="2"/>
       <c r="C12" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D12" t="s" s="2">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E12" s="2"/>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D13" t="s" s="2">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E13" s="2"/>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D14" t="s" s="2">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E14" s="2"/>
     </row>
@@ -757,7 +754,7 @@
         <v>31</v>
       </c>
       <c r="D2" t="s" s="2">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E2" t="s" s="2">
         <v>31</v>
@@ -772,10 +769,10 @@
         <v>34</v>
       </c>
       <c r="D3" t="s" s="2">
+        <v>59</v>
+      </c>
+      <c r="E3" t="s" s="2">
         <v>60</v>
-      </c>
-      <c r="E3" t="s" s="2">
-        <v>61</v>
       </c>
     </row>
     <row r="4">
@@ -787,7 +784,7 @@
         <v>34</v>
       </c>
       <c r="D4" t="s" s="2">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E4" s="2"/>
     </row>
@@ -800,7 +797,7 @@
         <v>34</v>
       </c>
       <c r="D5" t="s" s="2">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E5" s="2"/>
     </row>
@@ -813,7 +810,7 @@
         <v>34</v>
       </c>
       <c r="D6" t="s" s="2">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E6" s="2"/>
     </row>
@@ -826,33 +823,33 @@
         <v>34</v>
       </c>
       <c r="D7" t="s" s="2">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E7" s="2"/>
     </row>
     <row r="8">
       <c r="A8" t="s" s="2">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B8" s="2"/>
       <c r="C8" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D8" t="s" s="2">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E8" s="2"/>
     </row>
     <row r="9">
       <c r="A9" t="s" s="2">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B9" s="2"/>
       <c r="C9" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D9" t="s" s="2">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E9" s="2"/>
     </row>
@@ -865,7 +862,7 @@
         <v>34</v>
       </c>
       <c r="D10" t="s" s="2">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E10" s="2"/>
     </row>
@@ -878,7 +875,7 @@
         <v>34</v>
       </c>
       <c r="D11" t="s" s="2">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E11" s="2"/>
     </row>
@@ -891,111 +888,111 @@
         <v>34</v>
       </c>
       <c r="D12" t="s" s="2">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E12" s="2"/>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B13" s="2"/>
       <c r="C13" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D13" t="s" s="2">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E13" s="2"/>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B14" s="2"/>
       <c r="C14" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D14" t="s" s="2">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E14" s="2"/>
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B15" s="2"/>
       <c r="C15" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D15" t="s" s="2">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E15" s="2"/>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B16" s="2"/>
       <c r="C16" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D16" t="s" s="2">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E16" s="2"/>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B17" s="2"/>
       <c r="C17" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D17" t="s" s="2">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E17" s="2"/>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B18" s="2"/>
       <c r="C18" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D18" t="s" s="2">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E18" s="2"/>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B19" s="2"/>
       <c r="C19" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="D19" t="s" s="2">
         <v>82</v>
-      </c>
-      <c r="D19" t="s" s="2">
-        <v>83</v>
       </c>
       <c r="E19" s="2"/>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" t="s" s="2">
         <v>34</v>
       </c>
       <c r="D20" t="s" s="2">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E20" s="2"/>
     </row>

</xml_diff>